<commit_message>
se añadió horario y calnedario
</commit_message>
<xml_diff>
--- a/tercero/horario.xlsx
+++ b/tercero/horario.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb8fb80bea0f0cce/Desktop/uniiii/Uni2/universidad_git/tercero/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="192" documentId="8_{AA0B8A35-63F9-498F-8428-341B0363E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6C41048-BC90-46B1-AE01-BE446446D3F0}"/>
+  <xr:revisionPtr revIDLastSave="457" documentId="8_{AA0B8A35-63F9-498F-8428-341B0363E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E329319F-AEEB-4346-959F-3A7C0D7DE62D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7E10A3E1-B496-47EC-B443-F2FD5CDDA2E8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Horario" sheetId="1" r:id="rId1"/>
+    <sheet name="Calendario" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
   <si>
     <t>9:00-10:00</t>
   </si>
@@ -150,37 +150,181 @@
     <t>Diciembre</t>
   </si>
   <si>
-    <t>26 1 ª Entrega práctica</t>
-  </si>
-  <si>
-    <t>23 2 ª entrega práctica</t>
-  </si>
-  <si>
     <t>Enero</t>
   </si>
   <si>
-    <t>13 entrega final práctica</t>
-  </si>
-  <si>
-    <t>20 examen de to</t>
-  </si>
-  <si>
     <t>30 entrega ficha grupos</t>
   </si>
   <si>
     <t>.</t>
   </si>
   <si>
-    <t>2 entrega memoria práctica</t>
-  </si>
-  <si>
-    <t>9 entrega archivo práctica y código</t>
-  </si>
-  <si>
-    <t>25 examen de to</t>
-  </si>
-  <si>
-    <t>7 primer parcial</t>
+    <t>entrega Seguridad de las tecnologías</t>
+  </si>
+  <si>
+    <t>Seguridad de las tecnologías</t>
+  </si>
+  <si>
+    <t>Enunciado de "módulo de introducción a linux"</t>
+  </si>
+  <si>
+    <t>por confirmar</t>
+  </si>
+  <si>
+    <t>exámenes de sistemas operativos</t>
+  </si>
+  <si>
+    <t>Tercero</t>
+  </si>
+  <si>
+    <t>Segundo</t>
+  </si>
+  <si>
+    <t>Primero</t>
+  </si>
+  <si>
+    <t>Mates Discretas I</t>
+  </si>
+  <si>
+    <t>Mates Discretas II</t>
+  </si>
+  <si>
+    <t>3 Enunciado, "módulo de arquitectura e introducción al sistema operativo" SSOO</t>
+  </si>
+  <si>
+    <t>10 Ejercicio propuesto: Sistema de Ficheros SSOO</t>
+  </si>
+  <si>
+    <t>17 Enunciado, "módulo de ficheros" SSOO</t>
+  </si>
+  <si>
+    <t>16 Examen, confirmar con profe)?=)=)=)=   MD II</t>
+  </si>
+  <si>
+    <t>22 Examen, confirmar con profe)?=)=)=)=  MD I</t>
+  </si>
+  <si>
+    <t>21 Examen, confirmar con profe)?=)=)=)= SSOO</t>
+  </si>
+  <si>
+    <t>7 primer parcial, temas 1 y 2 IA</t>
+  </si>
+  <si>
+    <t>26 1 ª Entrega práctica    PDL</t>
+  </si>
+  <si>
+    <t>7 Ejercicio propuesto: Gestión de ficheros SSOO</t>
+  </si>
+  <si>
+    <t>14 Enunciado, "módulo de procesos" SSOO</t>
+  </si>
+  <si>
+    <t>28 Ejercicio propuesto: Gestión de memoria SSOO</t>
+  </si>
+  <si>
+    <t>18 Examen, confirmar con profe)?=)=)=)= SSOO</t>
+  </si>
+  <si>
+    <t>23 2 ª entrega práctica PDL</t>
+  </si>
+  <si>
+    <t>1 Examen Bloque I 42% ST</t>
+  </si>
+  <si>
+    <t>15 Ejercicios propuestos: Sincronización y Comunicación  SSOO</t>
+  </si>
+  <si>
+    <t>22 Examen Bloque II 42%  ST</t>
+  </si>
+  <si>
+    <t>16 Examen, confirmar con profe)?=)=)=)=  SSOO</t>
+  </si>
+  <si>
+    <t>9 entrega archivo práctica y código   IA</t>
+  </si>
+  <si>
+    <t>2 entrega memoria práctica  IA</t>
+  </si>
+  <si>
+    <t>5 Enunciado, "módulo de memoria"  SSOO</t>
+  </si>
+  <si>
+    <t>19 Enunciado, "módulo de sincronización y comunicación"  SSOO</t>
+  </si>
+  <si>
+    <t>26 MINISHELL   SSOO</t>
+  </si>
+  <si>
+    <t>20 examen de to  PDL</t>
+  </si>
+  <si>
+    <t>13 entrega final práctica  PDL</t>
+  </si>
+  <si>
+    <t>19 Examen Ordinario (en caso de no pasar la progresiva) 100%   ST</t>
+  </si>
+  <si>
+    <t>11 Examen, confirmar con profe)?=)=)=)=   MD I</t>
+  </si>
+  <si>
+    <t>25 examen de to  IA</t>
+  </si>
+  <si>
+    <t>12 Examen, confirmar con profe)?=)=)=)=   MD II</t>
+  </si>
+  <si>
+    <t>EC</t>
+  </si>
+  <si>
+    <t>MD II</t>
+  </si>
+  <si>
+    <t>MD I</t>
+  </si>
+  <si>
+    <t>SSOO</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>IA</t>
+  </si>
+  <si>
+    <t>PDL</t>
+  </si>
+  <si>
+    <t>17 Examen, confirmar con profe)?=)=)=)= EC</t>
+  </si>
+  <si>
+    <t>14 Examen, confirmar con profe)?=)=)=)= EC</t>
+  </si>
+  <si>
+    <t>PPS</t>
+  </si>
+  <si>
+    <t>LF</t>
+  </si>
+  <si>
+    <t>25 Examen, confirmar con profe)?=)=)=)= PPS</t>
+  </si>
+  <si>
+    <t>22 Examen, confirmar con profe)?=)=)=)= PPS</t>
+  </si>
+  <si>
+    <t>19 Examen, confirmar con profe)?=)=)=)=  LF</t>
+  </si>
+  <si>
+    <t>22 Parcial eliminatorio  LF</t>
+  </si>
+  <si>
+    <t>27 Parcial eliminatorio  LF</t>
+  </si>
+  <si>
+    <t>Algorítmica numérica</t>
+  </si>
+  <si>
+    <t>AN</t>
   </si>
 </sst>
 </file>
@@ -203,15 +347,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF92D050"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -254,8 +397,44 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -278,11 +457,235 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -310,48 +713,151 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF99"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -361,6 +867,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -680,6 +1190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2EF3B7-3EF8-4383-92A9-B24B7B5E299E}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="E5:P15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -734,21 +1245,21 @@
       <c r="F6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="19" t="s">
+      <c r="H6" s="19"/>
+      <c r="I6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="19"/>
+      <c r="J6" s="22"/>
       <c r="K6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="L6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="21"/>
+      <c r="M6" s="17"/>
       <c r="N6" s="11" t="s">
         <v>24</v>
       </c>
@@ -762,23 +1273,23 @@
       <c r="F7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="16"/>
-      <c r="I7" s="19" t="s">
+      <c r="H7" s="19"/>
+      <c r="I7" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="19"/>
+      <c r="J7" s="22"/>
       <c r="K7" s="2"/>
-      <c r="L7" s="13" t="s">
+      <c r="L7" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="13"/>
-      <c r="N7" s="21" t="s">
+      <c r="M7" s="18"/>
+      <c r="N7" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="O7" s="21"/>
+      <c r="O7" s="17"/>
       <c r="P7" s="3"/>
     </row>
     <row r="8" spans="5:16" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -786,21 +1297,21 @@
         <v>12</v>
       </c>
       <c r="F8" s="3"/>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="17"/>
-      <c r="I8" s="16" t="s">
+      <c r="H8" s="20"/>
+      <c r="I8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="16"/>
+      <c r="J8" s="19"/>
       <c r="K8" s="2"/>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
-      <c r="N8" s="21" t="s">
+      <c r="N8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="21"/>
+      <c r="O8" s="17"/>
       <c r="P8" s="11" t="s">
         <v>27</v>
       </c>
@@ -810,23 +1321,23 @@
         <v>13</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="19" t="s">
+      <c r="H9" s="19"/>
+      <c r="I9" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="19"/>
+      <c r="J9" s="22"/>
       <c r="K9" s="2"/>
-      <c r="L9" s="15" t="s">
+      <c r="L9" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="15"/>
-      <c r="N9" s="13" t="s">
+      <c r="M9" s="24"/>
+      <c r="N9" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="13"/>
+      <c r="O9" s="18"/>
       <c r="P9" s="3"/>
     </row>
     <row r="10" spans="5:16" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -834,17 +1345,17 @@
         <v>14</v>
       </c>
       <c r="F10" s="3"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="20" t="s">
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="20"/>
+      <c r="J10" s="23"/>
       <c r="K10" s="2"/>
-      <c r="L10" s="21" t="s">
+      <c r="L10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="21"/>
+      <c r="M10" s="17"/>
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
       <c r="P10" s="3"/>
@@ -871,6 +1382,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
     <mergeCell ref="N7:O7"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="N9:O9"/>
@@ -887,9 +1401,6 @@
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="L7:M7"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -897,10 +1408,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F2D5B9-8E16-4BF2-A85A-10B1240E3C08}">
-  <dimension ref="D3:M37"/>
+  <sheetPr codeName="Hoja2"/>
+  <dimension ref="D3:N41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="13" max="13" width="11.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
@@ -922,8 +1437,12 @@
       <c r="J3" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="4:13" x14ac:dyDescent="0.35">
+      <c r="L3" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="41"/>
+    </row>
+    <row r="4" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D4" s="14" t="s">
         <v>30</v>
       </c>
@@ -933,12 +1452,15 @@
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
       <c r="J4" s="14"/>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="22"/>
-    </row>
-    <row r="5" spans="4:13" x14ac:dyDescent="0.35">
+      <c r="M4" s="15"/>
+      <c r="N4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D5" s="3"/>
       <c r="E5" s="3">
         <v>8</v>
@@ -958,12 +1480,15 @@
       <c r="J5" s="3">
         <v>13</v>
       </c>
-      <c r="L5" s="24" t="s">
+      <c r="L5" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="24"/>
-    </row>
-    <row r="6" spans="4:13" x14ac:dyDescent="0.35">
+      <c r="M5" s="16"/>
+      <c r="N5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D6" s="3">
         <v>14</v>
       </c>
@@ -985,8 +1510,15 @@
       <c r="J6" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="4:13" x14ac:dyDescent="0.35">
+      <c r="L6" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="M6" s="26"/>
+      <c r="N6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D7" s="3">
         <v>21</v>
       </c>
@@ -1008,512 +1540,630 @@
       <c r="J7" s="3">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="4:13" x14ac:dyDescent="0.35">
+      <c r="L7" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="28"/>
+      <c r="N7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D8" s="3">
         <v>28</v>
       </c>
-      <c r="E8" s="3">
-        <v>29</v>
+      <c r="E8" s="27" t="s">
+        <v>39</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="10" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D10" s="14" t="s">
+    <row r="9" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="E9" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-    </row>
-    <row r="11" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3">
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="L11" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="M11" s="41"/>
+    </row>
+    <row r="12" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="3">
         <v>1</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H12" s="3">
         <v>2</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" s="3">
+        <v>4</v>
+      </c>
+      <c r="L12" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="M12" s="44"/>
+      <c r="N12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D13" s="3">
+        <v>5</v>
+      </c>
+      <c r="E13" s="34">
+        <v>6</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="32">
+        <v>8</v>
+      </c>
+      <c r="H13" s="3">
+        <v>9</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" s="3">
+        <v>11</v>
+      </c>
+      <c r="L13" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="M13" s="46"/>
+      <c r="N13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D14" s="3">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3">
+        <v>13</v>
+      </c>
+      <c r="F14" s="35">
+        <v>14</v>
+      </c>
+      <c r="G14" s="3">
+        <v>15</v>
+      </c>
+      <c r="H14" s="45" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="J14" s="3">
+        <v>18</v>
+      </c>
+      <c r="L14" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="M14" s="48"/>
+      <c r="N14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D15" s="3">
+        <v>19</v>
+      </c>
+      <c r="E15" s="3">
+        <v>20</v>
+      </c>
+      <c r="F15" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="H15" s="3">
+        <v>23</v>
+      </c>
+      <c r="I15" s="3">
+        <v>24</v>
+      </c>
+      <c r="J15" s="3">
+        <v>25</v>
+      </c>
+      <c r="L15" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="50"/>
+      <c r="N15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D16" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" s="3">
+        <v>28</v>
+      </c>
+      <c r="G16" s="3">
+        <v>29</v>
+      </c>
+      <c r="H16" s="3">
+        <v>30</v>
+      </c>
+      <c r="I16" s="3">
+        <v>31</v>
+      </c>
+      <c r="J16" s="3"/>
+      <c r="L16" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="M16" s="63"/>
+      <c r="N16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="4:14" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D18" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+    </row>
+    <row r="19" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3">
+        <v>1</v>
+      </c>
+      <c r="L19" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="M19" s="41"/>
+    </row>
+    <row r="20" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D20" s="3">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3">
         <v>3</v>
       </c>
-      <c r="J11" s="3">
+      <c r="F20" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D12" s="3">
+      <c r="G20" s="3">
         <v>5</v>
       </c>
-      <c r="E12" s="3">
+      <c r="H20" s="3">
         <v>6</v>
       </c>
-      <c r="F12" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="G12" s="3">
+      <c r="I20" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="J20" s="3">
         <v>8</v>
       </c>
-      <c r="H12" s="3">
+      <c r="L20" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="M20" s="42"/>
+      <c r="N20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D21" s="3">
         <v>9</v>
       </c>
-      <c r="I12" s="3">
+      <c r="E21" s="3">
         <v>10</v>
       </c>
-      <c r="J12" s="3">
+      <c r="F21" s="3">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D13" s="3">
+      <c r="G21" s="3">
         <v>12</v>
       </c>
-      <c r="E13" s="3">
+      <c r="H21" s="3">
         <v>13</v>
       </c>
-      <c r="F13" s="3">
+      <c r="I21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="J21" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D22" s="3">
+        <v>16</v>
+      </c>
+      <c r="E22" s="47" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" s="3">
+        <v>19</v>
+      </c>
+      <c r="H22" s="3">
+        <v>20</v>
+      </c>
+      <c r="I22" s="3">
+        <v>21</v>
+      </c>
+      <c r="J22" s="3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D23" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" s="3">
+        <v>24</v>
+      </c>
+      <c r="F23" s="49" t="s">
+        <v>88</v>
+      </c>
+      <c r="G23" s="3">
+        <v>26</v>
+      </c>
+      <c r="H23" s="3">
+        <v>27</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="J23" s="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="4:14" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="D24" s="3">
+        <v>30</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="26" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D26" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
+    </row>
+    <row r="27" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D27" s="3"/>
+      <c r="E27" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G27" s="3">
+        <v>3</v>
+      </c>
+      <c r="H27" s="3">
+        <v>4</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J27" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D28" s="3">
+        <v>7</v>
+      </c>
+      <c r="E28" s="3">
+        <v>8</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="G28" s="3">
+        <v>10</v>
+      </c>
+      <c r="H28" s="3">
+        <v>11</v>
+      </c>
+      <c r="I28" s="3">
+        <v>12</v>
+      </c>
+      <c r="J28" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D29" s="3">
         <v>14</v>
       </c>
-      <c r="G13" s="3">
+      <c r="E29" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="G29" s="3">
+        <v>17</v>
+      </c>
+      <c r="H29" s="3">
+        <v>18</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J29" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D30" s="55">
+        <v>21</v>
+      </c>
+      <c r="E30" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="F30" s="57">
+        <v>23</v>
+      </c>
+      <c r="G30" s="59">
+        <v>24</v>
+      </c>
+      <c r="H30" s="59">
+        <v>25</v>
+      </c>
+      <c r="I30" s="61" t="s">
+        <v>70</v>
+      </c>
+      <c r="J30" s="59">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D31" s="56"/>
+      <c r="E31" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="58"/>
+      <c r="G31" s="60"/>
+      <c r="H31" s="60"/>
+      <c r="I31" s="62"/>
+      <c r="J31" s="60"/>
+    </row>
+    <row r="32" spans="4:14" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="D32" s="3">
+        <v>28</v>
+      </c>
+      <c r="E32" s="3">
+        <v>29</v>
+      </c>
+      <c r="F32" s="3">
+        <v>30</v>
+      </c>
+      <c r="G32" s="3">
+        <v>31</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+    </row>
+    <row r="34" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D34" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="53"/>
+      <c r="I34" s="53"/>
+      <c r="J34" s="54"/>
+    </row>
+    <row r="35" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3">
+        <v>1</v>
+      </c>
+      <c r="I35" s="3">
+        <v>2</v>
+      </c>
+      <c r="J35" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="4:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D36" s="3">
+        <v>4</v>
+      </c>
+      <c r="E36" s="3">
+        <v>5</v>
+      </c>
+      <c r="F36" s="31">
+        <v>6</v>
+      </c>
+      <c r="G36" s="3">
+        <v>7</v>
+      </c>
+      <c r="H36" s="3">
+        <v>8</v>
+      </c>
+      <c r="I36" s="3">
+        <v>9</v>
+      </c>
+      <c r="J36" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D37" s="43" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37" s="45" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="G37" s="67" t="s">
+        <v>85</v>
+      </c>
+      <c r="H37" s="31">
         <v>15</v>
       </c>
-      <c r="H13" s="3">
+      <c r="I37" s="3">
         <v>16</v>
       </c>
-      <c r="I13" s="3">
+      <c r="J37" s="3">
         <v>17</v>
       </c>
-      <c r="J13" s="3">
+    </row>
+    <row r="38" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D38" s="72">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D14" s="3">
-        <v>19</v>
-      </c>
-      <c r="E14" s="3">
-        <v>20</v>
-      </c>
-      <c r="F14" s="3">
+      <c r="E38" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="F38" s="68" t="s">
+        <v>71</v>
+      </c>
+      <c r="G38" s="69">
         <v>21</v>
       </c>
-      <c r="G14" s="3">
-        <v>22</v>
-      </c>
-      <c r="H14" s="3">
+      <c r="H38" s="70" t="s">
+        <v>89</v>
+      </c>
+      <c r="I38" s="65">
         <v>23</v>
       </c>
-      <c r="I14" s="3">
+      <c r="J38" s="59">
         <v>24</v>
       </c>
-      <c r="J14" s="3">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="4:13" x14ac:dyDescent="0.35">
-      <c r="D15" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="3">
+    </row>
+    <row r="39" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D39" s="71"/>
+      <c r="E39" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="F39" s="68"/>
+      <c r="G39" s="69"/>
+      <c r="H39" s="70"/>
+      <c r="I39" s="58"/>
+      <c r="J39" s="60"/>
+    </row>
+    <row r="40" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D40" s="64" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40" s="3">
+        <v>26</v>
+      </c>
+      <c r="F40" s="66">
         <v>27</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G40" s="66">
         <v>28</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H40" s="66">
         <v>29</v>
       </c>
-      <c r="H15" s="3">
+      <c r="I40" s="3">
         <v>30</v>
       </c>
-      <c r="I15" s="3">
+      <c r="J40" s="3">
         <v>31</v>
       </c>
-      <c r="J15" s="3"/>
-    </row>
-    <row r="17" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D17" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-    </row>
-    <row r="18" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D19" s="3">
-        <v>2</v>
-      </c>
-      <c r="E19" s="3">
-        <v>3</v>
-      </c>
-      <c r="F19" s="3">
-        <v>4</v>
-      </c>
-      <c r="G19" s="3">
-        <v>5</v>
-      </c>
-      <c r="H19" s="3">
-        <v>6</v>
-      </c>
-      <c r="I19" s="3">
-        <v>7</v>
-      </c>
-      <c r="J19" s="3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D20" s="3">
-        <v>9</v>
-      </c>
-      <c r="E20" s="3">
-        <v>10</v>
-      </c>
-      <c r="F20" s="3">
-        <v>11</v>
-      </c>
-      <c r="G20" s="3">
-        <v>12</v>
-      </c>
-      <c r="H20" s="3">
-        <v>13</v>
-      </c>
-      <c r="I20" s="3">
-        <v>14</v>
-      </c>
-      <c r="J20" s="3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D21" s="3">
-        <v>16</v>
-      </c>
-      <c r="E21" s="3">
-        <v>17</v>
-      </c>
-      <c r="F21" s="3">
-        <v>18</v>
-      </c>
-      <c r="G21" s="3">
-        <v>19</v>
-      </c>
-      <c r="H21" s="3">
-        <v>20</v>
-      </c>
-      <c r="I21" s="3">
-        <v>21</v>
-      </c>
-      <c r="J21" s="3">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D22" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="3">
-        <v>24</v>
-      </c>
-      <c r="F22" s="3">
-        <v>25</v>
-      </c>
-      <c r="G22" s="3">
-        <v>26</v>
-      </c>
-      <c r="H22" s="3">
-        <v>27</v>
-      </c>
-      <c r="I22" s="3">
-        <v>28</v>
-      </c>
-      <c r="J22" s="3">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D23" s="3">
-        <v>30</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-    </row>
-    <row r="25" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D25" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-    </row>
-    <row r="26" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D26" s="3"/>
-      <c r="E26" s="3">
-        <v>1</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="G26" s="3">
-        <v>3</v>
-      </c>
-      <c r="H26" s="3">
-        <v>4</v>
-      </c>
-      <c r="I26" s="3">
-        <v>5</v>
-      </c>
-      <c r="J26" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D27" s="3">
-        <v>7</v>
-      </c>
-      <c r="E27" s="3">
-        <v>8</v>
-      </c>
-      <c r="F27" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="G27" s="3">
-        <v>10</v>
-      </c>
-      <c r="H27" s="3">
-        <v>11</v>
-      </c>
-      <c r="I27" s="3">
-        <v>12</v>
-      </c>
-      <c r="J27" s="3">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D28" s="3">
-        <v>14</v>
-      </c>
-      <c r="E28" s="3">
-        <v>15</v>
-      </c>
-      <c r="F28" s="3">
-        <v>16</v>
-      </c>
-      <c r="G28" s="3">
-        <v>17</v>
-      </c>
-      <c r="H28" s="3">
-        <v>18</v>
-      </c>
-      <c r="I28" s="3">
-        <v>19</v>
-      </c>
-      <c r="J28" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D29" s="3">
-        <v>21</v>
-      </c>
-      <c r="E29" s="3">
-        <v>22</v>
-      </c>
-      <c r="F29" s="3">
-        <v>23</v>
-      </c>
-      <c r="G29" s="3">
-        <v>24</v>
-      </c>
-      <c r="H29" s="3">
-        <v>25</v>
-      </c>
-      <c r="I29" s="3">
-        <v>26</v>
-      </c>
-      <c r="J29" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D30" s="3">
-        <v>28</v>
-      </c>
-      <c r="E30" s="3">
-        <v>29</v>
-      </c>
-      <c r="F30" s="3">
-        <v>30</v>
-      </c>
-      <c r="G30" s="3">
-        <v>31</v>
-      </c>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-    </row>
-    <row r="32" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D32" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-    </row>
-    <row r="33" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3">
-        <v>1</v>
-      </c>
-      <c r="I33" s="3">
-        <v>2</v>
-      </c>
-      <c r="J33" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D34" s="3">
-        <v>4</v>
-      </c>
-      <c r="E34" s="3">
-        <v>5</v>
-      </c>
-      <c r="F34" s="3">
-        <v>6</v>
-      </c>
-      <c r="G34" s="3">
-        <v>7</v>
-      </c>
-      <c r="H34" s="3">
-        <v>8</v>
-      </c>
-      <c r="I34" s="3">
-        <v>9</v>
-      </c>
-      <c r="J34" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D35" s="3">
-        <v>11</v>
-      </c>
-      <c r="E35" s="3">
-        <v>12</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G35" s="3">
-        <v>14</v>
-      </c>
-      <c r="H35" s="3">
-        <v>15</v>
-      </c>
-      <c r="I35" s="3">
-        <v>16</v>
-      </c>
-      <c r="J35" s="3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D36" s="3">
-        <v>18</v>
-      </c>
-      <c r="E36" s="3">
-        <v>19</v>
-      </c>
-      <c r="F36" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="G36" s="3">
-        <v>21</v>
-      </c>
-      <c r="H36" s="3">
-        <v>22</v>
-      </c>
-      <c r="I36" s="3">
-        <v>23</v>
-      </c>
-      <c r="J36" s="3">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D37" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="E37" s="3">
-        <v>26</v>
-      </c>
-      <c r="F37" s="3">
-        <v>27</v>
-      </c>
-      <c r="G37" s="3">
-        <v>28</v>
-      </c>
-      <c r="H37" s="3">
-        <v>29</v>
-      </c>
-      <c r="I37" s="3">
-        <v>30</v>
-      </c>
-      <c r="J37" s="3">
-        <v>31</v>
-      </c>
-    </row>
+    </row>
+    <row r="41" spans="4:10" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="D25:J25"/>
+  <mergeCells count="30">
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="D34:J34"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="J30:J31"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="D26:J26"/>
     <mergeCell ref="L4:M4"/>
-    <mergeCell ref="D32:J32"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="D4:J4"/>
-    <mergeCell ref="D10:J10"/>
-    <mergeCell ref="D17:J17"/>
+    <mergeCell ref="D11:J11"/>
+    <mergeCell ref="D18:J18"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
actualización SSOO y LF
</commit_message>
<xml_diff>
--- a/tercero/horario.xlsx
+++ b/tercero/horario.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb8fb80bea0f0cce/Desktop/uniiii/Uni2/universidad_git/tercero/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="457" documentId="8_{AA0B8A35-63F9-498F-8428-341B0363E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E329319F-AEEB-4346-959F-3A7C0D7DE62D}"/>
+  <xr:revisionPtr revIDLastSave="460" documentId="8_{AA0B8A35-63F9-498F-8428-341B0363E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79C6F170-F1A4-4A75-B77D-2544DBEB9FF9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7E10A3E1-B496-47EC-B443-F2FD5CDDA2E8}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="96">
   <si>
     <t>9:00-10:00</t>
   </si>
@@ -306,9 +306,6 @@
     <t>LF</t>
   </si>
   <si>
-    <t>25 Examen, confirmar con profe)?=)=)=)= PPS</t>
-  </si>
-  <si>
     <t>22 Examen, confirmar con profe)?=)=)=)= PPS</t>
   </si>
   <si>
@@ -325,6 +322,12 @@
   </si>
   <si>
     <t>AN</t>
+  </si>
+  <si>
+    <t>Primer semestre</t>
+  </si>
+  <si>
+    <t>25 Examen PPS</t>
   </si>
 </sst>
 </file>
@@ -685,7 +688,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -714,47 +717,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -767,29 +731,80 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -808,44 +823,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1245,21 +1251,21 @@
       <c r="F6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="19"/>
-      <c r="I6" s="22" t="s">
+      <c r="H6" s="69"/>
+      <c r="I6" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="22"/>
+      <c r="J6" s="68"/>
       <c r="K6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="17"/>
+      <c r="M6" s="66"/>
       <c r="N6" s="11" t="s">
         <v>24</v>
       </c>
@@ -1273,23 +1279,23 @@
       <c r="F7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="19"/>
-      <c r="I7" s="22" t="s">
+      <c r="H7" s="69"/>
+      <c r="I7" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="22"/>
+      <c r="J7" s="68"/>
       <c r="K7" s="2"/>
-      <c r="L7" s="18" t="s">
+      <c r="L7" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="18"/>
-      <c r="N7" s="17" t="s">
+      <c r="M7" s="67"/>
+      <c r="N7" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="O7" s="17"/>
+      <c r="O7" s="66"/>
       <c r="P7" s="3"/>
     </row>
     <row r="8" spans="5:16" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1297,21 +1303,21 @@
         <v>12</v>
       </c>
       <c r="F8" s="3"/>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="20"/>
-      <c r="I8" s="19" t="s">
+      <c r="H8" s="71"/>
+      <c r="I8" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="19"/>
+      <c r="J8" s="69"/>
       <c r="K8" s="2"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="17" t="s">
+      <c r="L8" s="37"/>
+      <c r="M8" s="37"/>
+      <c r="N8" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="17"/>
+      <c r="O8" s="66"/>
       <c r="P8" s="11" t="s">
         <v>27</v>
       </c>
@@ -1321,23 +1327,23 @@
         <v>13</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="19"/>
-      <c r="I9" s="22" t="s">
+      <c r="H9" s="69"/>
+      <c r="I9" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="22"/>
+      <c r="J9" s="68"/>
       <c r="K9" s="2"/>
-      <c r="L9" s="24" t="s">
+      <c r="L9" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="24"/>
-      <c r="N9" s="18" t="s">
+      <c r="M9" s="73"/>
+      <c r="N9" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="18"/>
+      <c r="O9" s="67"/>
       <c r="P9" s="3"/>
     </row>
     <row r="10" spans="5:16" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1345,19 +1351,19 @@
         <v>14</v>
       </c>
       <c r="F10" s="3"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="23" t="s">
+      <c r="G10" s="72"/>
+      <c r="H10" s="72"/>
+      <c r="I10" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="23"/>
+      <c r="J10" s="70"/>
       <c r="K10" s="2"/>
-      <c r="L10" s="17" t="s">
+      <c r="L10" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="17"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
+      <c r="M10" s="66"/>
+      <c r="N10" s="37"/>
+      <c r="O10" s="37"/>
       <c r="P10" s="3"/>
     </row>
     <row r="12" spans="5:16" x14ac:dyDescent="0.35">
@@ -1382,25 +1388,25 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="L8:M8"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="N7:O7"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="N10:O10"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I10:J10"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H10"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:M8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1409,12 +1415,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F2D5B9-8E16-4BF2-A85A-10B1240E3C08}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="D3:N41"/>
+  <dimension ref="D1:N41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="13" max="13" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="L1" s="36" t="s">
+        <v>94</v>
+      </c>
+      <c r="M1" s="36"/>
+    </row>
     <row r="3" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D3" s="3" t="s">
         <v>10</v>
@@ -1437,25 +1449,25 @@
       <c r="J3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="41" t="s">
+      <c r="L3" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="M3" s="41"/>
+      <c r="M3" s="40"/>
     </row>
     <row r="4" spans="4:14" x14ac:dyDescent="0.35">
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="L4" s="15" t="s">
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+      <c r="L4" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="15"/>
+      <c r="M4" s="46"/>
       <c r="N4" t="s">
         <v>83</v>
       </c>
@@ -1480,10 +1492,10 @@
       <c r="J5" s="3">
         <v>13</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="16"/>
+      <c r="M5" s="47"/>
       <c r="N5" t="s">
         <v>82</v>
       </c>
@@ -1510,10 +1522,10 @@
       <c r="J6" s="3">
         <v>20</v>
       </c>
-      <c r="L6" s="26" t="s">
+      <c r="L6" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="M6" s="26"/>
+      <c r="M6" s="38"/>
       <c r="N6" t="s">
         <v>81</v>
       </c>
@@ -1540,10 +1552,10 @@
       <c r="J7" s="3">
         <v>27</v>
       </c>
-      <c r="L7" s="28" t="s">
+      <c r="L7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="28"/>
+      <c r="M7" s="39"/>
       <c r="N7" t="s">
         <v>80</v>
       </c>
@@ -1552,10 +1564,10 @@
       <c r="D8" s="3">
         <v>28</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="25" t="s">
+      <c r="F8" s="14" t="s">
         <v>37</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -1566,38 +1578,38 @@
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="4:14" x14ac:dyDescent="0.35">
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="17" t="s">
         <v>41</v>
       </c>
       <c r="F9" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="40" t="s">
+      <c r="L9" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="M9" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" spans="4:14" x14ac:dyDescent="0.35">
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="L11" s="41" t="s">
+      <c r="E11" s="37"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="37"/>
+      <c r="L11" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="M11" s="41"/>
+      <c r="M11" s="40"/>
     </row>
     <row r="12" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="33"/>
+      <c r="F12" s="20"/>
       <c r="G12" s="3">
         <v>1</v>
       </c>
@@ -1610,10 +1622,10 @@
       <c r="J12" s="3">
         <v>4</v>
       </c>
-      <c r="L12" s="44" t="s">
+      <c r="L12" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="M12" s="44"/>
+      <c r="M12" s="42"/>
       <c r="N12" t="s">
         <v>78</v>
       </c>
@@ -1622,13 +1634,13 @@
       <c r="D13" s="3">
         <v>5</v>
       </c>
-      <c r="E13" s="34">
+      <c r="E13" s="21">
         <v>6</v>
       </c>
-      <c r="F13" s="36" t="s">
+      <c r="F13" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="19">
         <v>8</v>
       </c>
       <c r="H13" s="3">
@@ -1640,10 +1652,10 @@
       <c r="J13" s="3">
         <v>11</v>
       </c>
-      <c r="L13" s="46" t="s">
+      <c r="L13" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="46"/>
+      <c r="M13" s="43"/>
       <c r="N13" t="s">
         <v>77</v>
       </c>
@@ -1655,13 +1667,13 @@
       <c r="E14" s="3">
         <v>13</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="22">
         <v>14</v>
       </c>
       <c r="G14" s="3">
         <v>15</v>
       </c>
-      <c r="H14" s="45" t="s">
+      <c r="H14" s="29" t="s">
         <v>52</v>
       </c>
       <c r="I14" s="8" t="s">
@@ -1670,10 +1682,10 @@
       <c r="J14" s="3">
         <v>18</v>
       </c>
-      <c r="L14" s="48" t="s">
+      <c r="L14" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="M14" s="48"/>
+      <c r="M14" s="44"/>
       <c r="N14" t="s">
         <v>86</v>
       </c>
@@ -1685,10 +1697,10 @@
       <c r="E15" s="3">
         <v>20</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="G15" s="43" t="s">
+      <c r="G15" s="28" t="s">
         <v>53</v>
       </c>
       <c r="H15" s="3">
@@ -1700,10 +1712,10 @@
       <c r="J15" s="3">
         <v>25</v>
       </c>
-      <c r="L15" s="50" t="s">
+      <c r="L15" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="50"/>
+      <c r="M15" s="45"/>
       <c r="N15" t="s">
         <v>87</v>
       </c>
@@ -1712,8 +1724,8 @@
       <c r="D16" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="51" t="s">
-        <v>92</v>
+      <c r="E16" s="32" t="s">
+        <v>91</v>
       </c>
       <c r="F16" s="3">
         <v>28</v>
@@ -1728,25 +1740,25 @@
         <v>31</v>
       </c>
       <c r="J16" s="3"/>
-      <c r="L16" s="63" t="s">
+      <c r="L16" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="M16" s="50"/>
+      <c r="N16" t="s">
         <v>93</v>
-      </c>
-      <c r="M16" s="63"/>
-      <c r="N16" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="4:14" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="4:14" x14ac:dyDescent="0.35">
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
     </row>
     <row r="19" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D19" s="3"/>
@@ -1758,10 +1770,10 @@
       <c r="J19" s="3">
         <v>1</v>
       </c>
-      <c r="L19" s="41" t="s">
+      <c r="L19" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="M19" s="41"/>
+      <c r="M19" s="40"/>
     </row>
     <row r="20" spans="4:14" x14ac:dyDescent="0.35">
       <c r="D20" s="3">
@@ -1785,10 +1797,10 @@
       <c r="J20" s="3">
         <v>8</v>
       </c>
-      <c r="L20" s="42" t="s">
+      <c r="L20" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="M20" s="42"/>
+      <c r="M20" s="41"/>
       <c r="N20" t="s">
         <v>79</v>
       </c>
@@ -1820,10 +1832,10 @@
       <c r="D22" s="3">
         <v>16</v>
       </c>
-      <c r="E22" s="47" t="s">
+      <c r="E22" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="F22" s="26" t="s">
         <v>60</v>
       </c>
       <c r="G22" s="3">
@@ -1846,8 +1858,8 @@
       <c r="E23" s="3">
         <v>24</v>
       </c>
-      <c r="F23" s="49" t="s">
-        <v>88</v>
+      <c r="F23" s="31" t="s">
+        <v>95</v>
       </c>
       <c r="G23" s="3">
         <v>26</v>
@@ -1874,19 +1886,19 @@
       <c r="J24" s="3"/>
     </row>
     <row r="26" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="37"/>
     </row>
     <row r="27" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D27" s="3"/>
-      <c r="E27" s="38" t="s">
+      <c r="E27" s="25" t="s">
         <v>62</v>
       </c>
       <c r="F27" s="13" t="s">
@@ -1935,7 +1947,7 @@
       <c r="E29" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F29" s="39" t="s">
+      <c r="F29" s="26" t="s">
         <v>65</v>
       </c>
       <c r="G29" s="3">
@@ -1952,38 +1964,38 @@
       </c>
     </row>
     <row r="30" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D30" s="55">
+      <c r="D30" s="61">
         <v>21</v>
       </c>
-      <c r="E30" s="38" t="s">
+      <c r="E30" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="F30" s="57">
+      <c r="F30" s="63">
         <v>23</v>
       </c>
-      <c r="G30" s="59">
+      <c r="G30" s="48">
         <v>24</v>
       </c>
-      <c r="H30" s="59">
+      <c r="H30" s="48">
         <v>25</v>
       </c>
-      <c r="I30" s="61" t="s">
+      <c r="I30" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="J30" s="59">
+      <c r="J30" s="48">
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="4:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D31" s="56"/>
-      <c r="E31" s="51" t="s">
-        <v>91</v>
-      </c>
-      <c r="F31" s="58"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="60"/>
-      <c r="I31" s="62"/>
-      <c r="J31" s="60"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="F31" s="57"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="65"/>
+      <c r="J31" s="49"/>
     </row>
     <row r="32" spans="4:14" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="D32" s="3">
@@ -2003,15 +2015,15 @@
       <c r="J32" s="3"/>
     </row>
     <row r="34" spans="4:10" x14ac:dyDescent="0.35">
-      <c r="D34" s="52" t="s">
+      <c r="D34" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="E34" s="53"/>
-      <c r="F34" s="53"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="53"/>
-      <c r="I34" s="53"/>
-      <c r="J34" s="54"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="59"/>
+      <c r="I34" s="59"/>
+      <c r="J34" s="60"/>
     </row>
     <row r="35" spans="4:10" x14ac:dyDescent="0.35">
       <c r="D35" s="3"/>
@@ -2035,7 +2047,7 @@
       <c r="E36" s="3">
         <v>5</v>
       </c>
-      <c r="F36" s="31">
+      <c r="F36" s="18">
         <v>6</v>
       </c>
       <c r="G36" s="3">
@@ -2052,19 +2064,19 @@
       </c>
     </row>
     <row r="37" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D37" s="43" t="s">
+      <c r="D37" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="E37" s="45" t="s">
+      <c r="E37" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="37" t="s">
+      <c r="F37" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="G37" s="67" t="s">
+      <c r="G37" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="H37" s="31">
+      <c r="H37" s="18">
         <v>15</v>
       </c>
       <c r="I37" s="3">
@@ -2075,53 +2087,53 @@
       </c>
     </row>
     <row r="38" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D38" s="72">
+      <c r="D38" s="51">
         <v>18</v>
       </c>
-      <c r="E38" s="38" t="s">
+      <c r="E38" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="F38" s="68" t="s">
+      <c r="F38" s="53" t="s">
         <v>71</v>
       </c>
-      <c r="G38" s="69">
+      <c r="G38" s="54">
         <v>21</v>
       </c>
-      <c r="H38" s="70" t="s">
+      <c r="H38" s="55" t="s">
+        <v>88</v>
+      </c>
+      <c r="I38" s="56">
+        <v>23</v>
+      </c>
+      <c r="J38" s="48">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D39" s="52"/>
+      <c r="E39" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="I38" s="65">
-        <v>23</v>
-      </c>
-      <c r="J38" s="59">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D39" s="71"/>
-      <c r="E39" s="51" t="s">
-        <v>90</v>
-      </c>
-      <c r="F39" s="68"/>
-      <c r="G39" s="69"/>
-      <c r="H39" s="70"/>
-      <c r="I39" s="58"/>
-      <c r="J39" s="60"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="55"/>
+      <c r="I39" s="57"/>
+      <c r="J39" s="49"/>
     </row>
     <row r="40" spans="4:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D40" s="64" t="s">
+      <c r="D40" s="33" t="s">
         <v>75</v>
       </c>
       <c r="E40" s="3">
         <v>26</v>
       </c>
-      <c r="F40" s="66">
+      <c r="F40" s="34">
         <v>27</v>
       </c>
-      <c r="G40" s="66">
+      <c r="G40" s="34">
         <v>28</v>
       </c>
-      <c r="H40" s="66">
+      <c r="H40" s="34">
         <v>29</v>
       </c>
       <c r="I40" s="3">
@@ -2133,7 +2145,7 @@
     </row>
     <row r="41" spans="4:10" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="J38:J39"/>
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="D38:D39"/>
@@ -2148,22 +2160,23 @@
     <mergeCell ref="H30:H31"/>
     <mergeCell ref="I30:I31"/>
     <mergeCell ref="J30:J31"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="D26:J26"/>
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="L20:M20"/>
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="L13:M13"/>
     <mergeCell ref="L14:M14"/>
     <mergeCell ref="L15:M15"/>
-    <mergeCell ref="D26:J26"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L1:M1"/>
     <mergeCell ref="D4:J4"/>
     <mergeCell ref="D11:J11"/>
     <mergeCell ref="D18:J18"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>